<commit_message>
Minor reference to Trello added
</commit_message>
<xml_diff>
--- a/Homework 03 - Product Backlog.xlsx
+++ b/Homework 03 - Product Backlog.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9c7c63b8d3e1e1c/School/4 - Info Sys Proj Mgmt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="193" documentId="11_F25DC773A252ABDACC1048EEF9187A645BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C5C746D-7292-434A-B249-83A6283682E7}"/>
+  <xr:revisionPtr revIDLastSave="199" documentId="11_F25DC773A252ABDACC1048EEF9187A645BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC2D0237-243C-4A6F-B55C-2C8576B23B18}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="112">
   <si>
     <t>Feature</t>
   </si>
@@ -358,6 +358,9 @@
   </si>
   <si>
     <t>Add report export functionality</t>
+  </si>
+  <si>
+    <t>This Excel sheet is the complete product backlog, while the Trello board functions as a high-level representation.</t>
   </si>
 </sst>
 </file>
@@ -393,8 +396,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -421,6 +427,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -698,7 +708,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
@@ -1289,8 +1299,18 @@
         <v>110</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B55" s="1"/>
+      <c r="C55" s="1"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B25:B56">
+  <mergeCells count="1">
+    <mergeCell ref="A55:C55"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B25:B54 B56">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>